<commit_message>
[WIP] Ajout du mapping MOS-Annuaire (#188)
* add mappings

* rm old mapping

* document bug

* upodate bake and nos to false

* update version

* add nos

* add bake

* test mapping

* test org mapping

* test 2

* update

* add mapping org

* update liste profils

* update mappings and practitionerrole heritage

* correct errors

* update Practitioner and PractitionerRole mappings

* add generate

* correct errors

* update mappings 034de7512c471e122cd3d84b679193979814469f
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-as-address-extended.xlsx
+++ b/main/ig/StructureDefinition-as-address-extended.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1111" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1108" uniqueCount="281">
   <si>
     <t>Property</t>
   </si>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-04-08T12:53:48+00:00</t>
+    <t>2024-04-09T07:46:55+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -484,10 +484,19 @@
     <t>Address.line.id</t>
   </si>
   <si>
+    <t>xml:id (or equivalent in JSON)</t>
+  </si>
+  <si>
+    <t>unique id for the element within a resource (for internal references)</t>
+  </si>
+  <si>
     <t>Address.line.extension</t>
   </si>
   <si>
-    <t>N/A</t>
+    <t>Extension</t>
+  </si>
+  <si>
+    <t>An Extension</t>
   </si>
   <si>
     <t>Address.line.extension:careOf</t>
@@ -622,6 +631,9 @@
     <t>Extension.url</t>
   </si>
   <si>
+    <t>N/A</t>
+  </si>
+  <si>
     <t>Address.line.extension:streetNameType.value[x]</t>
   </si>
   <si>
@@ -631,7 +643,7 @@
     <t>Value of extension</t>
   </si>
   <si>
-    <t>Value of extension - must be one of a constrained set of the data types (see [Extensibility](http://hl7.org/fhir/R4/extensibility.html) for a list).</t>
+    <t>Value of extension - must be one of a constrained set of the data types (see [Extensibility](http://hl7.org/fhir/extensibility.html) for a list).</t>
   </si>
   <si>
     <t>https://mos.esante.gouv.fr/NOS/JDV_J103-TypeVoie-RASS/FHIR/JDV-J103-TypeVoie-RASS</t>
@@ -698,6 +710,9 @@
   </si>
   <si>
     <t>Primitive value for string</t>
+  </si>
+  <si>
+    <t>The actual value</t>
   </si>
   <si>
     <t>1048576</t>
@@ -2296,10 +2311,10 @@
         <v>90</v>
       </c>
       <c r="L10" t="s" s="2">
-        <v>91</v>
+        <v>152</v>
       </c>
       <c r="M10" t="s" s="2">
-        <v>92</v>
+        <v>153</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
@@ -2368,7 +2383,7 @@
         <v>77</v>
       </c>
       <c r="AL10" t="s" s="2">
-        <v>94</v>
+        <v>77</v>
       </c>
       <c r="AM10" t="s" s="2">
         <v>77</v>
@@ -2379,14 +2394,14 @@
     </row>
     <row r="11" hidden="true">
       <c r="A11" t="s" s="2">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="B11" t="s" s="2">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" t="s" s="2">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11" t="s" s="2">
@@ -2408,14 +2423,12 @@
         <v>97</v>
       </c>
       <c r="L11" t="s" s="2">
-        <v>98</v>
+        <v>155</v>
       </c>
       <c r="M11" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="N11" t="s" s="2">
-        <v>100</v>
-      </c>
+        <v>156</v>
+      </c>
+      <c r="N11" s="2"/>
       <c r="O11" s="2"/>
       <c r="P11" t="s" s="2">
         <v>77</v>
@@ -2454,9 +2467,7 @@
       <c r="AB11" t="s" s="2">
         <v>101</v>
       </c>
-      <c r="AC11" t="s" s="2">
-        <v>102</v>
-      </c>
+      <c r="AC11" s="2"/>
       <c r="AD11" t="s" s="2">
         <v>77</v>
       </c>
@@ -2473,7 +2484,7 @@
         <v>79</v>
       </c>
       <c r="AI11" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="AJ11" t="s" s="2">
         <v>105</v>
@@ -2482,7 +2493,7 @@
         <v>77</v>
       </c>
       <c r="AL11" t="s" s="2">
-        <v>153</v>
+        <v>77</v>
       </c>
       <c r="AM11" t="s" s="2">
         <v>77</v>
@@ -2493,13 +2504,13 @@
     </row>
     <row r="12" hidden="true">
       <c r="A12" t="s" s="2">
+        <v>157</v>
+      </c>
+      <c r="B12" t="s" s="2">
         <v>154</v>
       </c>
-      <c r="B12" t="s" s="2">
-        <v>152</v>
-      </c>
       <c r="C12" t="s" s="2">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="D12" t="s" s="2">
         <v>77</v>
@@ -2521,13 +2532,13 @@
         <v>77</v>
       </c>
       <c r="K12" t="s" s="2">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="L12" t="s" s="2">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="M12" t="s" s="2">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
@@ -2596,7 +2607,7 @@
         <v>77</v>
       </c>
       <c r="AL12" t="s" s="2">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="AM12" t="s" s="2">
         <v>77</v>
@@ -2607,13 +2618,13 @@
     </row>
     <row r="13" hidden="true">
       <c r="A13" t="s" s="2">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B13" t="s" s="2">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C13" t="s" s="2">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="D13" t="s" s="2">
         <v>77</v>
@@ -2635,13 +2646,13 @@
         <v>77</v>
       </c>
       <c r="K13" t="s" s="2">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="L13" t="s" s="2">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="M13" t="s" s="2">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
@@ -2710,7 +2721,7 @@
         <v>77</v>
       </c>
       <c r="AL13" t="s" s="2">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="AM13" t="s" s="2">
         <v>77</v>
@@ -2721,13 +2732,13 @@
     </row>
     <row r="14" hidden="true">
       <c r="A14" t="s" s="2">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="B14" t="s" s="2">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C14" t="s" s="2">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="D14" t="s" s="2">
         <v>77</v>
@@ -2749,13 +2760,13 @@
         <v>77</v>
       </c>
       <c r="K14" t="s" s="2">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="L14" t="s" s="2">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="M14" t="s" s="2">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
@@ -2824,7 +2835,7 @@
         <v>77</v>
       </c>
       <c r="AL14" t="s" s="2">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="AM14" t="s" s="2">
         <v>77</v>
@@ -2835,13 +2846,13 @@
     </row>
     <row r="15" hidden="true">
       <c r="A15" t="s" s="2">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B15" t="s" s="2">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C15" t="s" s="2">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="D15" t="s" s="2">
         <v>77</v>
@@ -2863,13 +2874,13 @@
         <v>77</v>
       </c>
       <c r="K15" t="s" s="2">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="L15" t="s" s="2">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="M15" t="s" s="2">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="N15" s="2"/>
       <c r="O15" s="2"/>
@@ -2938,7 +2949,7 @@
         <v>77</v>
       </c>
       <c r="AL15" t="s" s="2">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="AM15" t="s" s="2">
         <v>77</v>
@@ -2949,13 +2960,13 @@
     </row>
     <row r="16" hidden="true">
       <c r="A16" t="s" s="2">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B16" t="s" s="2">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C16" t="s" s="2">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="D16" t="s" s="2">
         <v>77</v>
@@ -2977,13 +2988,13 @@
         <v>77</v>
       </c>
       <c r="K16" t="s" s="2">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="L16" t="s" s="2">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="M16" t="s" s="2">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="N16" s="2"/>
       <c r="O16" s="2"/>
@@ -3052,7 +3063,7 @@
         <v>77</v>
       </c>
       <c r="AL16" t="s" s="2">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="AM16" t="s" s="2">
         <v>77</v>
@@ -3063,10 +3074,10 @@
     </row>
     <row r="17" hidden="true">
       <c r="A17" t="s" s="2">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B17" t="s" s="2">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" t="s" s="2">
@@ -3175,14 +3186,14 @@
     </row>
     <row r="18" hidden="true">
       <c r="A18" t="s" s="2">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B18" t="s" s="2">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" t="s" s="2">
-        <v>96</v>
+        <v>77</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" t="s" s="2">
@@ -3204,14 +3215,12 @@
         <v>97</v>
       </c>
       <c r="L18" t="s" s="2">
-        <v>98</v>
+        <v>155</v>
       </c>
       <c r="M18" t="s" s="2">
-        <v>99</v>
-      </c>
-      <c r="N18" t="s" s="2">
-        <v>100</v>
-      </c>
+        <v>156</v>
+      </c>
+      <c r="N18" s="2"/>
       <c r="O18" s="2"/>
       <c r="P18" t="s" s="2">
         <v>77</v>
@@ -3269,7 +3278,7 @@
         <v>79</v>
       </c>
       <c r="AI18" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="AJ18" t="s" s="2">
         <v>105</v>
@@ -3278,7 +3287,7 @@
         <v>77</v>
       </c>
       <c r="AL18" t="s" s="2">
-        <v>153</v>
+        <v>77</v>
       </c>
       <c r="AM18" t="s" s="2">
         <v>77</v>
@@ -3289,10 +3298,10 @@
     </row>
     <row r="19" hidden="true">
       <c r="A19" t="s" s="2">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B19" t="s" s="2">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" t="s" s="2">
@@ -3315,16 +3324,16 @@
         <v>77</v>
       </c>
       <c r="K19" t="s" s="2">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="L19" t="s" s="2">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="M19" t="s" s="2">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="N19" t="s" s="2">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="O19" s="2"/>
       <c r="P19" t="s" s="2">
@@ -3332,7 +3341,7 @@
       </c>
       <c r="Q19" s="2"/>
       <c r="R19" t="s" s="2">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="S19" t="s" s="2">
         <v>77</v>
@@ -3374,7 +3383,7 @@
         <v>77</v>
       </c>
       <c r="AF19" t="s" s="2">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="AG19" t="s" s="2">
         <v>89</v>
@@ -3392,7 +3401,7 @@
         <v>77</v>
       </c>
       <c r="AL19" t="s" s="2">
-        <v>153</v>
+        <v>199</v>
       </c>
       <c r="AM19" t="s" s="2">
         <v>77</v>
@@ -3403,10 +3412,10 @@
     </row>
     <row r="20" hidden="true">
       <c r="A20" t="s" s="2">
-        <v>196</v>
+        <v>200</v>
       </c>
       <c r="B20" t="s" s="2">
-        <v>197</v>
+        <v>201</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" t="s" s="2">
@@ -3432,10 +3441,10 @@
         <v>90</v>
       </c>
       <c r="L20" t="s" s="2">
-        <v>198</v>
+        <v>202</v>
       </c>
       <c r="M20" t="s" s="2">
-        <v>199</v>
+        <v>203</v>
       </c>
       <c r="N20" s="2"/>
       <c r="O20" s="2"/>
@@ -3466,7 +3475,7 @@
       </c>
       <c r="Y20" s="2"/>
       <c r="Z20" t="s" s="2">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="AA20" t="s" s="2">
         <v>77</v>
@@ -3484,7 +3493,7 @@
         <v>77</v>
       </c>
       <c r="AF20" t="s" s="2">
-        <v>201</v>
+        <v>205</v>
       </c>
       <c r="AG20" t="s" s="2">
         <v>78</v>
@@ -3493,7 +3502,7 @@
         <v>89</v>
       </c>
       <c r="AI20" t="s" s="2">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="AJ20" t="s" s="2">
         <v>85</v>
@@ -3502,7 +3511,7 @@
         <v>77</v>
       </c>
       <c r="AL20" t="s" s="2">
-        <v>153</v>
+        <v>199</v>
       </c>
       <c r="AM20" t="s" s="2">
         <v>77</v>
@@ -3513,13 +3522,13 @@
     </row>
     <row r="21" hidden="true">
       <c r="A21" t="s" s="2">
-        <v>202</v>
+        <v>206</v>
       </c>
       <c r="B21" t="s" s="2">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C21" t="s" s="2">
-        <v>203</v>
+        <v>207</v>
       </c>
       <c r="D21" t="s" s="2">
         <v>77</v>
@@ -3541,13 +3550,13 @@
         <v>77</v>
       </c>
       <c r="K21" t="s" s="2">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="L21" t="s" s="2">
-        <v>205</v>
+        <v>209</v>
       </c>
       <c r="M21" t="s" s="2">
-        <v>206</v>
+        <v>210</v>
       </c>
       <c r="N21" s="2"/>
       <c r="O21" s="2"/>
@@ -3616,7 +3625,7 @@
         <v>77</v>
       </c>
       <c r="AL21" t="s" s="2">
-        <v>207</v>
+        <v>211</v>
       </c>
       <c r="AM21" t="s" s="2">
         <v>77</v>
@@ -3627,13 +3636,13 @@
     </row>
     <row r="22" hidden="true">
       <c r="A22" t="s" s="2">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="B22" t="s" s="2">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C22" t="s" s="2">
-        <v>209</v>
+        <v>213</v>
       </c>
       <c r="D22" t="s" s="2">
         <v>77</v>
@@ -3655,13 +3664,13 @@
         <v>77</v>
       </c>
       <c r="K22" t="s" s="2">
-        <v>210</v>
+        <v>214</v>
       </c>
       <c r="L22" t="s" s="2">
-        <v>211</v>
+        <v>215</v>
       </c>
       <c r="M22" t="s" s="2">
-        <v>212</v>
+        <v>216</v>
       </c>
       <c r="N22" s="2"/>
       <c r="O22" s="2"/>
@@ -3730,7 +3739,7 @@
         <v>77</v>
       </c>
       <c r="AL22" t="s" s="2">
-        <v>213</v>
+        <v>217</v>
       </c>
       <c r="AM22" t="s" s="2">
         <v>77</v>
@@ -3741,13 +3750,13 @@
     </row>
     <row r="23" hidden="true">
       <c r="A23" t="s" s="2">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="B23" t="s" s="2">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="C23" t="s" s="2">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="D23" t="s" s="2">
         <v>77</v>
@@ -3769,13 +3778,13 @@
         <v>77</v>
       </c>
       <c r="K23" t="s" s="2">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="L23" t="s" s="2">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="M23" t="s" s="2">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="N23" s="2"/>
       <c r="O23" s="2"/>
@@ -3855,10 +3864,10 @@
     </row>
     <row r="24" hidden="true">
       <c r="A24" t="s" s="2">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="B24" t="s" s="2">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" t="s" s="2">
@@ -3884,10 +3893,10 @@
         <v>90</v>
       </c>
       <c r="L24" t="s" s="2">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="M24" t="s" s="2">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="N24" s="2"/>
       <c r="O24" s="2"/>
@@ -3911,7 +3920,7 @@
         <v>77</v>
       </c>
       <c r="W24" t="s" s="2">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="X24" t="s" s="2">
         <v>77</v>
@@ -3938,7 +3947,7 @@
         <v>77</v>
       </c>
       <c r="AF24" t="s" s="2">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="AG24" t="s" s="2">
         <v>78</v>
@@ -3967,14 +3976,14 @@
     </row>
     <row r="25" hidden="true">
       <c r="A25" t="s" s="2">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="B25" t="s" s="2">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" t="s" s="2">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="E25" s="2"/>
       <c r="F25" t="s" s="2">
@@ -3996,10 +4005,10 @@
         <v>90</v>
       </c>
       <c r="L25" t="s" s="2">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="M25" t="s" s="2">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="N25" s="2"/>
       <c r="O25" s="2"/>
@@ -4014,7 +4023,7 @@
         <v>77</v>
       </c>
       <c r="T25" t="s" s="2">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="U25" t="s" s="2">
         <v>77</v>
@@ -4050,7 +4059,7 @@
         <v>77</v>
       </c>
       <c r="AF25" t="s" s="2">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="AG25" t="s" s="2">
         <v>78</v>
@@ -4065,28 +4074,28 @@
         <v>85</v>
       </c>
       <c r="AK25" t="s" s="2">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="AL25" t="s" s="2">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="AM25" t="s" s="2">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="AN25" t="s" s="2">
-        <v>231</v>
+        <v>236</v>
       </c>
     </row>
     <row r="26" hidden="true">
       <c r="A26" t="s" s="2">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="B26" t="s" s="2">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" t="s" s="2">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="E26" s="2"/>
       <c r="F26" t="s" s="2">
@@ -4108,13 +4117,13 @@
         <v>90</v>
       </c>
       <c r="L26" t="s" s="2">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="M26" t="s" s="2">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="N26" t="s" s="2">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="O26" s="2"/>
       <c r="P26" t="s" s="2">
@@ -4128,7 +4137,7 @@
         <v>77</v>
       </c>
       <c r="T26" t="s" s="2">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="U26" t="s" s="2">
         <v>77</v>
@@ -4144,7 +4153,7 @@
       </c>
       <c r="Y26" s="2"/>
       <c r="Z26" t="s" s="2">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="AA26" t="s" s="2">
         <v>77</v>
@@ -4162,7 +4171,7 @@
         <v>77</v>
       </c>
       <c r="AF26" t="s" s="2">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="AG26" t="s" s="2">
         <v>78</v>
@@ -4177,10 +4186,10 @@
         <v>85</v>
       </c>
       <c r="AK26" t="s" s="2">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="AL26" t="s" s="2">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="AM26" t="s" s="2">
         <v>77</v>
@@ -4191,14 +4200,14 @@
     </row>
     <row r="27" hidden="true">
       <c r="A27" t="s" s="2">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="B27" t="s" s="2">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" t="s" s="2">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="E27" s="2"/>
       <c r="F27" t="s" s="2">
@@ -4220,10 +4229,10 @@
         <v>90</v>
       </c>
       <c r="L27" t="s" s="2">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="M27" t="s" s="2">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="N27" s="2"/>
       <c r="O27" s="2"/>
@@ -4274,7 +4283,7 @@
         <v>77</v>
       </c>
       <c r="AF27" t="s" s="2">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="AG27" t="s" s="2">
         <v>78</v>
@@ -4289,28 +4298,28 @@
         <v>85</v>
       </c>
       <c r="AK27" t="s" s="2">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="AL27" t="s" s="2">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="AM27" t="s" s="2">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="AN27" t="s" s="2">
-        <v>248</v>
+        <v>253</v>
       </c>
     </row>
     <row r="28" hidden="true">
       <c r="A28" t="s" s="2">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="B28" t="s" s="2">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" t="s" s="2">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="E28" s="2"/>
       <c r="F28" t="s" s="2">
@@ -4332,10 +4341,10 @@
         <v>90</v>
       </c>
       <c r="L28" t="s" s="2">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="M28" t="s" s="2">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="N28" s="2"/>
       <c r="O28" s="2"/>
@@ -4350,7 +4359,7 @@
         <v>77</v>
       </c>
       <c r="T28" t="s" s="2">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="U28" t="s" s="2">
         <v>77</v>
@@ -4386,7 +4395,7 @@
         <v>77</v>
       </c>
       <c r="AF28" t="s" s="2">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="AG28" t="s" s="2">
         <v>78</v>
@@ -4401,24 +4410,24 @@
         <v>85</v>
       </c>
       <c r="AK28" t="s" s="2">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="AL28" t="s" s="2">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="AM28" t="s" s="2">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="AN28" t="s" s="2">
-        <v>257</v>
+        <v>262</v>
       </c>
     </row>
     <row r="29" hidden="true">
       <c r="A29" t="s" s="2">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="B29" t="s" s="2">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" t="s" s="2">
@@ -4444,13 +4453,13 @@
         <v>90</v>
       </c>
       <c r="L29" t="s" s="2">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="M29" t="s" s="2">
-        <v>260</v>
+        <v>265</v>
       </c>
       <c r="N29" t="s" s="2">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="O29" s="2"/>
       <c r="P29" t="s" s="2">
@@ -4480,7 +4489,7 @@
       </c>
       <c r="Y29" s="2"/>
       <c r="Z29" t="s" s="2">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="AA29" t="s" s="2">
         <v>77</v>
@@ -4498,7 +4507,7 @@
         <v>77</v>
       </c>
       <c r="AF29" t="s" s="2">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="AG29" t="s" s="2">
         <v>78</v>
@@ -4513,24 +4522,24 @@
         <v>85</v>
       </c>
       <c r="AK29" t="s" s="2">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="AL29" t="s" s="2">
-        <v>264</v>
+        <v>269</v>
       </c>
       <c r="AM29" t="s" s="2">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="AN29" t="s" s="2">
-        <v>266</v>
+        <v>271</v>
       </c>
     </row>
     <row r="30" hidden="true">
       <c r="A30" t="s" s="2">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="B30" t="s" s="2">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" t="s" s="2">
@@ -4553,17 +4562,17 @@
         <v>112</v>
       </c>
       <c r="K30" t="s" s="2">
-        <v>268</v>
+        <v>273</v>
       </c>
       <c r="L30" t="s" s="2">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="M30" t="s" s="2">
-        <v>270</v>
+        <v>275</v>
       </c>
       <c r="N30" s="2"/>
       <c r="O30" t="s" s="2">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="P30" t="s" s="2">
         <v>77</v>
@@ -4576,43 +4585,43 @@
         <v>77</v>
       </c>
       <c r="T30" t="s" s="2">
+        <v>277</v>
+      </c>
+      <c r="U30" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="V30" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="W30" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="X30" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Y30" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="Z30" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AA30" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AB30" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AC30" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AD30" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AE30" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AF30" t="s" s="2">
         <v>272</v>
-      </c>
-      <c r="U30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="V30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="W30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="X30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Y30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="Z30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AA30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AB30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AC30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AD30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AE30" t="s" s="2">
-        <v>77</v>
-      </c>
-      <c r="AF30" t="s" s="2">
-        <v>267</v>
       </c>
       <c r="AG30" t="s" s="2">
         <v>78</v>
@@ -4627,13 +4636,13 @@
         <v>85</v>
       </c>
       <c r="AK30" t="s" s="2">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="AL30" t="s" s="2">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="AM30" t="s" s="2">
-        <v>275</v>
+        <v>280</v>
       </c>
       <c r="AN30" t="s" s="2">
         <v>77</v>

</xml_diff>

<commit_message>
update pays (#258) bf438dee20be9f4e3e19c5e8d20aca326e9c2d29
</commit_message>
<xml_diff>
--- a/main/ig/StructureDefinition-as-address-extended.xlsx
+++ b/main/ig/StructureDefinition-as-address-extended.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2025-02-11T13:37:59+00:00</t>
+    <t>2025-02-11T14:09:44+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -883,7 +883,7 @@
     <t>ISO 3166 3 letter codes can be used in place of a human readable country name.</t>
   </si>
   <si>
-    <t>https://mos.esante.gouv.fr/NOS/JDV_J74-Pays-RASS/FHIR/JDV-J74-Pays-RASS</t>
+    <t>https://mos.esante.gouv.fr/NOS/JDV_J256-Pays/FHIR/JDV-J256-Pays</t>
   </si>
   <si>
     <t>XAD.6</t>

</xml_diff>